<commit_message>
fix(ci): optimize GitHub Actions workflows, fix cache dependency, update mobile build and test reports
</commit_message>
<xml_diff>
--- a/all-excel-reports/02_SpareGrow_Appium_Mobile_E2E_Test_Report.xlsx
+++ b/all-excel-reports/02_SpareGrow_Appium_Mobile_E2E_Test_Report.xlsx
@@ -24,7 +24,7 @@
     <t>SPAREGROW MOBILE APP – APPIUM E2E AUTOMATION TEST REPORT (NODE.JS)</t>
   </si>
   <si>
-    <t>Generated: 2/8/2026, 2:44:20 pm | Framework: Appium / WebDriverIO (Node.js) | Target: Android APK</t>
+    <t>Generated: 6/8/2026, 9:08:55 am | Framework: Appium / WebDriverIO (Node.js) | Target: Android APK</t>
   </si>
   <si>
     <t>100.0%</t>
@@ -153,7 +153,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>2026-08-02 09:14:20</t>
+    <t>2026-08-06 03:38:55</t>
   </si>
   <si>
     <t>APK file integrity and size valid (&gt;2MB)</t>
@@ -3291,7 +3291,7 @@
     <t>CLOSED / RESOLVED</t>
   </si>
   <si>
-    <t>2/8/2026</t>
+    <t>6/8/2026</t>
   </si>
 </sst>
 </file>

</xml_diff>